<commit_message>
v1.0.2: Finalize Gemini pacing shield and ignore output_docs
</commit_message>
<xml_diff>
--- a/output_docs/doc1.xlsx
+++ b/output_docs/doc1.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H79"/>
+  <dimension ref="A1:G78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -452,11 +452,6 @@
           <t>Rate</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
-        <is>
-          <t>Discount</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="n">
@@ -478,7 +473,6 @@
       </c>
       <c r="F2" t="inlineStr"/>
       <c r="G2" t="inlineStr"/>
-      <c r="H2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="n">
@@ -500,7 +494,6 @@
       </c>
       <c r="F3" t="inlineStr"/>
       <c r="G3" t="inlineStr"/>
-      <c r="H3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="n">
@@ -522,7 +515,6 @@
       </c>
       <c r="F4" t="inlineStr"/>
       <c r="G4" t="inlineStr"/>
-      <c r="H4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="n">
@@ -544,7 +536,6 @@
       </c>
       <c r="F5" t="inlineStr"/>
       <c r="G5" t="inlineStr"/>
-      <c r="H5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="n">
@@ -566,7 +557,6 @@
       </c>
       <c r="F6" t="inlineStr"/>
       <c r="G6" t="inlineStr"/>
-      <c r="H6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="n">
@@ -588,7 +578,6 @@
       </c>
       <c r="F7" t="inlineStr"/>
       <c r="G7" t="inlineStr"/>
-      <c r="H7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="n">
@@ -610,7 +599,6 @@
       </c>
       <c r="F8" t="inlineStr"/>
       <c r="G8" t="inlineStr"/>
-      <c r="H8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="n">
@@ -632,7 +620,6 @@
       </c>
       <c r="F9" t="inlineStr"/>
       <c r="G9" t="inlineStr"/>
-      <c r="H9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="n">
@@ -654,7 +641,6 @@
       </c>
       <c r="F10" t="inlineStr"/>
       <c r="G10" t="inlineStr"/>
-      <c r="H10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="n">
@@ -676,7 +662,6 @@
       </c>
       <c r="F11" t="inlineStr"/>
       <c r="G11" t="inlineStr"/>
-      <c r="H11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="n">
@@ -698,7 +683,6 @@
       </c>
       <c r="F12" t="inlineStr"/>
       <c r="G12" t="inlineStr"/>
-      <c r="H12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="n">
@@ -720,7 +704,6 @@
       </c>
       <c r="F13" t="inlineStr"/>
       <c r="G13" t="inlineStr"/>
-      <c r="H13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="n">
@@ -742,7 +725,6 @@
       </c>
       <c r="F14" t="inlineStr"/>
       <c r="G14" t="inlineStr"/>
-      <c r="H14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="n">
@@ -764,7 +746,6 @@
       <c r="G15" t="n">
         <v>440</v>
       </c>
-      <c r="H15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="n">
@@ -786,7 +767,6 @@
       <c r="G16" t="n">
         <v>176</v>
       </c>
-      <c r="H16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="n">
@@ -808,7 +788,6 @@
       <c r="G17" t="n">
         <v>385</v>
       </c>
-      <c r="H17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="n">
@@ -830,7 +809,6 @@
       <c r="G18" t="n">
         <v>44</v>
       </c>
-      <c r="H18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="n">
@@ -852,7 +830,6 @@
       <c r="G19" t="n">
         <v>110</v>
       </c>
-      <c r="H19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="n">
@@ -874,7 +851,6 @@
       <c r="G20" t="n">
         <v>264</v>
       </c>
-      <c r="H20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="n">
@@ -896,7 +872,6 @@
       <c r="G21" t="n">
         <v>77</v>
       </c>
-      <c r="H21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="n">
@@ -918,9 +893,6 @@
       <c r="G22" t="n">
         <v>220</v>
       </c>
-      <c r="H22" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="23">
       <c r="A23" t="n">
@@ -936,9 +908,6 @@
       <c r="F23" t="n">
         <v>220</v>
       </c>
-      <c r="H23" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="24">
       <c r="A24" t="n">
@@ -960,9 +929,6 @@
       <c r="G24" t="n">
         <v>110</v>
       </c>
-      <c r="H24" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="25">
       <c r="A25" t="n">
@@ -984,9 +950,6 @@
       <c r="G25" t="n">
         <v>66</v>
       </c>
-      <c r="H25" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="26">
       <c r="A26" t="n">
@@ -1008,9 +971,6 @@
       <c r="G26" t="n">
         <v>165</v>
       </c>
-      <c r="H26" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="n">
@@ -1032,9 +992,6 @@
       <c r="G27" t="n">
         <v>31.5</v>
       </c>
-      <c r="H27" t="n">
-        <v>6.3</v>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="n">
@@ -1056,9 +1013,6 @@
       <c r="G28" t="n">
         <v>12</v>
       </c>
-      <c r="H28" t="n">
-        <v>2.4</v>
-      </c>
     </row>
     <row r="29">
       <c r="A29" t="n">
@@ -1080,9 +1034,6 @@
       <c r="G29" t="n">
         <v>12</v>
       </c>
-      <c r="H29" t="n">
-        <v>1.92</v>
-      </c>
     </row>
     <row r="30">
       <c r="A30" t="n">
@@ -1104,9 +1055,6 @@
       <c r="G30" t="n">
         <v>16.5</v>
       </c>
-      <c r="H30" t="n">
-        <v>3.3</v>
-      </c>
     </row>
     <row r="31">
       <c r="A31" t="n">
@@ -1128,9 +1076,6 @@
       <c r="G31" t="n">
         <v>201</v>
       </c>
-      <c r="H31" t="n">
-        <v>80.40000000000001</v>
-      </c>
     </row>
     <row r="32">
       <c r="A32" t="n">
@@ -1152,9 +1097,6 @@
       <c r="G32" t="n">
         <v>5.32</v>
       </c>
-      <c r="H32" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="33">
       <c r="A33" t="n">
@@ -1176,9 +1118,6 @@
       <c r="G33" t="n">
         <v>5.32</v>
       </c>
-      <c r="H33" t="n">
-        <v>0</v>
-      </c>
     </row>
     <row r="34">
       <c r="A34" t="n">
@@ -1200,9 +1139,6 @@
       <c r="G34" t="n">
         <v>4</v>
       </c>
-      <c r="H34" t="n">
-        <v>0.64</v>
-      </c>
     </row>
     <row r="35">
       <c r="A35" t="n">
@@ -1224,9 +1160,6 @@
       <c r="G35" t="n">
         <v>2</v>
       </c>
-      <c r="H35" t="n">
-        <v>0.11</v>
-      </c>
     </row>
     <row r="36">
       <c r="A36" t="n">
@@ -1234,21 +1167,20 @@
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Std Ac Room-2-Dw8</t>
+          <t>Vitcee Fort</t>
         </is>
       </c>
       <c r="C36" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr"/>
       <c r="F36" t="n">
-        <v>660</v>
+        <v>445.32</v>
       </c>
       <c r="G36" t="n">
-        <v>220</v>
-      </c>
-      <c r="H36" t="inlineStr"/>
+        <v>445.32</v>
+      </c>
     </row>
     <row r="37">
       <c r="A37" t="n">
@@ -1256,21 +1188,20 @@
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>Vitcee Fort</t>
+          <t>10 Ml Syringe</t>
         </is>
       </c>
       <c r="C37" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr"/>
       <c r="F37" t="n">
-        <v>445.32</v>
+        <v>126</v>
       </c>
       <c r="G37" t="n">
-        <v>445.32</v>
-      </c>
-      <c r="H37" t="inlineStr"/>
+        <v>31.5</v>
+      </c>
     </row>
     <row r="38">
       <c r="A38" t="n">
@@ -1278,21 +1209,20 @@
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>10 Ml Syringe</t>
+          <t>Drip Set Dis</t>
         </is>
       </c>
       <c r="C38" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr"/>
       <c r="F38" t="n">
-        <v>126</v>
+        <v>201</v>
       </c>
       <c r="G38" t="n">
-        <v>31.5</v>
-      </c>
-      <c r="H38" t="inlineStr"/>
+        <v>201</v>
+      </c>
     </row>
     <row r="39">
       <c r="A39" t="n">
@@ -1300,21 +1230,20 @@
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>2 Ml Syringe Dis</t>
+          <t>Easy Fix</t>
         </is>
       </c>
       <c r="C39" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr"/>
       <c r="F39" t="n">
-        <v>48</v>
+        <v>56</v>
       </c>
       <c r="G39" t="n">
-        <v>12</v>
-      </c>
-      <c r="H39" t="inlineStr"/>
+        <v>56</v>
+      </c>
     </row>
     <row r="40">
       <c r="A40" t="n">
@@ -1322,7 +1251,7 @@
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>Drip Set Dis</t>
+          <t>Iv Cannula 24g Dis</t>
         </is>
       </c>
       <c r="C40" t="n">
@@ -1331,12 +1260,11 @@
       <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr"/>
       <c r="F40" t="n">
-        <v>201</v>
+        <v>191.25</v>
       </c>
       <c r="G40" t="n">
-        <v>201</v>
-      </c>
-      <c r="H40" t="inlineStr"/>
+        <v>191.25</v>
+      </c>
     </row>
     <row r="41">
       <c r="A41" t="n">
@@ -1344,21 +1272,20 @@
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>Easy Fix</t>
+          <t>Abiflu 75 Cap</t>
         </is>
       </c>
       <c r="C41" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr"/>
       <c r="F41" t="n">
-        <v>56</v>
+        <v>280.38</v>
       </c>
       <c r="G41" t="n">
-        <v>56</v>
-      </c>
-      <c r="H41" t="inlineStr"/>
+        <v>46.73</v>
+      </c>
     </row>
     <row r="42">
       <c r="A42" t="n">
@@ -1366,21 +1293,20 @@
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>Iv Cannula 24g Dis</t>
+          <t>Bidel 100mg Inj Bidel 100mg Inj</t>
         </is>
       </c>
       <c r="C42" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D42" t="inlineStr"/>
       <c r="E42" t="inlineStr"/>
       <c r="F42" t="n">
-        <v>191.25</v>
+        <v>1073.82</v>
       </c>
       <c r="G42" t="n">
-        <v>191.25</v>
-      </c>
-      <c r="H42" t="inlineStr"/>
+        <v>536.91</v>
+      </c>
     </row>
     <row r="43">
       <c r="A43" t="n">
@@ -1388,87 +1314,83 @@
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Needle 16*1 1/2</t>
+          <t>Espentral - 40</t>
         </is>
       </c>
       <c r="C43" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="D43" t="inlineStr"/>
       <c r="E43" t="inlineStr"/>
       <c r="F43" t="n">
-        <v>21.28</v>
+        <v>270</v>
       </c>
       <c r="G43" t="n">
-        <v>5.32</v>
-      </c>
-      <c r="H43" t="inlineStr"/>
+        <v>135</v>
+      </c>
     </row>
     <row r="44">
       <c r="A44" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>Abiflu 75 Cap</t>
+          <t>Fexolite M Tab</t>
         </is>
       </c>
       <c r="C44" t="n">
-        <v>6</v>
-      </c>
-      <c r="D44" t="inlineStr"/>
-      <c r="E44" t="inlineStr"/>
-      <c r="F44" t="n">
-        <v>280.38</v>
-      </c>
-      <c r="G44" t="n">
-        <v>46.73</v>
-      </c>
-      <c r="H44" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="D44" t="n">
+        <v>98</v>
+      </c>
+      <c r="E44" t="n">
+        <v>98</v>
+      </c>
+      <c r="F44" t="inlineStr"/>
+      <c r="G44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>Bidel 100mg Inj Bidel 100mg Inj</t>
+          <t>Livi 300mg Tab</t>
         </is>
       </c>
       <c r="C45" t="n">
-        <v>2</v>
-      </c>
-      <c r="D45" t="inlineStr"/>
-      <c r="E45" t="inlineStr"/>
-      <c r="F45" t="n">
-        <v>1073.82</v>
-      </c>
-      <c r="G45" t="n">
-        <v>536.91</v>
-      </c>
-      <c r="H45" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="D45" t="n">
+        <v>192</v>
+      </c>
+      <c r="E45" t="n">
+        <v>192</v>
+      </c>
+      <c r="F45" t="inlineStr"/>
+      <c r="G45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>Espentral - 40</t>
+          <t>Menis - Sb Inj</t>
         </is>
       </c>
       <c r="C46" t="n">
-        <v>2</v>
-      </c>
-      <c r="D46" t="inlineStr"/>
-      <c r="E46" t="inlineStr"/>
-      <c r="F46" t="n">
-        <v>270</v>
-      </c>
-      <c r="G46" t="n">
-        <v>135</v>
-      </c>
-      <c r="H46" t="inlineStr"/>
+        <v>3</v>
+      </c>
+      <c r="D46" t="n">
+        <v>3093.75</v>
+      </c>
+      <c r="E46" t="n">
+        <v>3093.75</v>
+      </c>
+      <c r="F46" t="inlineStr"/>
+      <c r="G46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="n">
@@ -1476,21 +1398,20 @@
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>Fexolite M Tab</t>
+          <t>Meronorm 1gm Inj</t>
         </is>
       </c>
       <c r="C47" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D47" t="n">
-        <v>16.34</v>
+        <v>1331.24</v>
       </c>
       <c r="E47" t="n">
-        <v>98.04000000000001</v>
+        <v>1331.24</v>
       </c>
       <c r="F47" t="inlineStr"/>
       <c r="G47" t="inlineStr"/>
-      <c r="H47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="n">
@@ -1498,21 +1419,20 @@
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>Livi 300mg Tab</t>
+          <t>Normal Saline 100ml</t>
         </is>
       </c>
       <c r="C48" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D48" t="n">
-        <v>32</v>
+        <v>90.44</v>
       </c>
       <c r="E48" t="n">
-        <v>192</v>
+        <v>90.44</v>
       </c>
       <c r="F48" t="inlineStr"/>
       <c r="G48" t="inlineStr"/>
-      <c r="H48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="n">
@@ -1520,21 +1440,20 @@
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>Menis - Sb Inj</t>
+          <t>Normal Saline 100ml</t>
         </is>
       </c>
       <c r="C49" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D49" t="n">
-        <v>1031.25</v>
+        <v>180</v>
       </c>
       <c r="E49" t="n">
-        <v>3093.75</v>
+        <v>180</v>
       </c>
       <c r="F49" t="inlineStr"/>
       <c r="G49" t="inlineStr"/>
-      <c r="H49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="n">
@@ -1542,21 +1461,20 @@
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>Meronorm 1gm Inj</t>
+          <t>Normal Saline Ivf</t>
         </is>
       </c>
       <c r="C50" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D50" t="n">
-        <v>665.62</v>
+        <v>94.55</v>
       </c>
       <c r="E50" t="n">
-        <v>1331.24</v>
+        <v>94.55</v>
       </c>
       <c r="F50" t="inlineStr"/>
       <c r="G50" t="inlineStr"/>
-      <c r="H50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="n">
@@ -1564,21 +1482,20 @@
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>Normal Saline 100ml</t>
+          <t>Piximole 100 Ml</t>
         </is>
       </c>
       <c r="C51" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D51" t="n">
-        <v>45.22</v>
+        <v>897</v>
       </c>
       <c r="E51" t="n">
-        <v>90.44</v>
+        <v>897</v>
       </c>
       <c r="F51" t="inlineStr"/>
       <c r="G51" t="inlineStr"/>
-      <c r="H51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="n">
@@ -1586,21 +1503,20 @@
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>Normal Saline 100ml</t>
+          <t>Polybion Inj</t>
         </is>
       </c>
       <c r="C52" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="D52" t="n">
-        <v>45.22</v>
+        <v>25.78</v>
       </c>
       <c r="E52" t="n">
-        <v>180.88</v>
+        <v>25.78</v>
       </c>
       <c r="F52" t="inlineStr"/>
       <c r="G52" t="inlineStr"/>
-      <c r="H52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="n">
@@ -1608,21 +1524,20 @@
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Normal Saline Ivf</t>
+          <t>Ringer Lactate Ivf</t>
         </is>
       </c>
       <c r="C53" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D53" t="n">
-        <v>94.55</v>
+        <v>138.78</v>
       </c>
       <c r="E53" t="n">
-        <v>94.55</v>
+        <v>138.78</v>
       </c>
       <c r="F53" t="inlineStr"/>
       <c r="G53" t="inlineStr"/>
-      <c r="H53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="n">
@@ -1630,21 +1545,20 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Piximole 100 Ml</t>
+          <t>Bidel 100mg Inj</t>
         </is>
       </c>
       <c r="C54" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="D54" t="n">
-        <v>299</v>
+        <v>1073.82</v>
       </c>
       <c r="E54" t="n">
-        <v>897</v>
+        <v>1073.82</v>
       </c>
       <c r="F54" t="inlineStr"/>
       <c r="G54" t="inlineStr"/>
-      <c r="H54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="n">
@@ -1652,21 +1566,20 @@
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Polybion Inj</t>
+          <t>Espentral - 40</t>
         </is>
       </c>
       <c r="C55" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D55" t="n">
-        <v>25.78</v>
+        <v>270</v>
       </c>
       <c r="E55" t="n">
-        <v>25.78</v>
+        <v>270</v>
       </c>
       <c r="F55" t="inlineStr"/>
       <c r="G55" t="inlineStr"/>
-      <c r="H55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="n">
@@ -1674,21 +1587,20 @@
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Ringer Lactate Ivf</t>
+          <t>Menis - Sb Inj</t>
         </is>
       </c>
       <c r="C56" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D56" t="n">
-        <v>69.39</v>
+        <v>3093.74</v>
       </c>
       <c r="E56" t="n">
-        <v>138.78</v>
+        <v>3093.74</v>
       </c>
       <c r="F56" t="inlineStr"/>
       <c r="G56" t="inlineStr"/>
-      <c r="H56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="n">
@@ -1696,21 +1608,20 @@
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Bidel 100mg Inj</t>
+          <t>Normal Saline 100ml</t>
         </is>
       </c>
       <c r="C57" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="D57" t="n">
-        <v>536.91</v>
+        <v>135</v>
       </c>
       <c r="E57" t="n">
-        <v>1073.82</v>
+        <v>135</v>
       </c>
       <c r="F57" t="inlineStr"/>
       <c r="G57" t="inlineStr"/>
-      <c r="H57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="n">
@@ -1718,21 +1629,20 @@
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Espentral - 40</t>
+          <t>Abiflu 75 Cap</t>
         </is>
       </c>
       <c r="C58" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D58" t="n">
-        <v>135</v>
+        <v>280.4</v>
       </c>
       <c r="E58" t="n">
-        <v>270</v>
+        <v>280.4</v>
       </c>
       <c r="F58" t="inlineStr"/>
       <c r="G58" t="inlineStr"/>
-      <c r="H58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="n">
@@ -1740,21 +1650,20 @@
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>Normal Saline 100ml</t>
+          <t>Doxy 1 Tab</t>
         </is>
       </c>
       <c r="C59" t="n">
-        <v>3</v>
+        <v>14</v>
       </c>
       <c r="D59" t="n">
-        <v>45.22</v>
+        <v>158.48</v>
       </c>
       <c r="E59" t="n">
-        <v>135.66</v>
+        <v>158.48</v>
       </c>
       <c r="F59" t="inlineStr"/>
       <c r="G59" t="inlineStr"/>
-      <c r="H59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="n">
@@ -1762,21 +1671,20 @@
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>Abiflu 75 Cap</t>
+          <t>Emeset Inj 2 Ml</t>
         </is>
       </c>
       <c r="C60" t="n">
-        <v>6</v>
+        <v>2</v>
       </c>
       <c r="D60" t="n">
-        <v>46.73</v>
+        <v>25.44</v>
       </c>
       <c r="E60" t="n">
-        <v>280.38</v>
+        <v>25.44</v>
       </c>
       <c r="F60" t="inlineStr"/>
       <c r="G60" t="inlineStr"/>
-      <c r="H60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="n">
@@ -1784,21 +1692,20 @@
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>Doxy 1 Tab</t>
+          <t>Farotic 200</t>
         </is>
       </c>
       <c r="C61" t="n">
-        <v>14</v>
+        <v>21</v>
       </c>
       <c r="D61" t="n">
-        <v>11.32</v>
+        <v>2362.5</v>
       </c>
       <c r="E61" t="n">
-        <v>158.48</v>
+        <v>2362.5</v>
       </c>
       <c r="F61" t="inlineStr"/>
       <c r="G61" t="inlineStr"/>
-      <c r="H61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="n">
@@ -1806,21 +1713,20 @@
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>Emeset Inj 2 Ml</t>
+          <t>Fexolite M Tab</t>
         </is>
       </c>
       <c r="C62" t="n">
-        <v>2</v>
+        <v>6</v>
       </c>
       <c r="D62" t="n">
-        <v>12.72</v>
+        <v>16.34</v>
       </c>
       <c r="E62" t="n">
-        <v>25.44</v>
+        <v>98.04000000000001</v>
       </c>
       <c r="F62" t="inlineStr"/>
       <c r="G62" t="inlineStr"/>
-      <c r="H62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="n">
@@ -1828,21 +1734,20 @@
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>Farotic 200</t>
+          <t>Fexolite M Tab</t>
         </is>
       </c>
       <c r="C63" t="n">
-        <v>21</v>
+        <v>7</v>
       </c>
       <c r="D63" t="n">
-        <v>112.5</v>
+        <v>16.34</v>
       </c>
       <c r="E63" t="n">
-        <v>2362.5</v>
+        <v>114.38</v>
       </c>
       <c r="F63" t="inlineStr"/>
       <c r="G63" t="inlineStr"/>
-      <c r="H63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="n">
@@ -1850,21 +1755,20 @@
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>Fexolite M Tab</t>
+          <t>Piximole 100 Ml</t>
         </is>
       </c>
       <c r="C64" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="D64" t="n">
-        <v>16.34</v>
+        <v>299</v>
       </c>
       <c r="E64" t="n">
-        <v>114.38</v>
+        <v>299</v>
       </c>
       <c r="F64" t="inlineStr"/>
       <c r="G64" t="inlineStr"/>
-      <c r="H64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="n">
@@ -1872,21 +1776,20 @@
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>Piximole 100 Ml</t>
+          <t>Probotix Cap</t>
         </is>
       </c>
       <c r="C65" t="n">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="D65" t="n">
-        <v>299</v>
+        <v>16.91</v>
       </c>
       <c r="E65" t="n">
-        <v>299</v>
+        <v>236.74</v>
       </c>
       <c r="F65" t="inlineStr"/>
       <c r="G65" t="inlineStr"/>
-      <c r="H65" t="inlineStr"/>
     </row>
     <row r="66">
       <c r="A66" t="n">
@@ -1894,21 +1797,20 @@
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>Probotix Cap</t>
+          <t>Supralite Os Syp</t>
         </is>
       </c>
       <c r="C66" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="D66" t="n">
-        <v>16.91</v>
+        <v>309</v>
       </c>
       <c r="E66" t="n">
-        <v>236.74</v>
+        <v>309</v>
       </c>
       <c r="F66" t="inlineStr"/>
       <c r="G66" t="inlineStr"/>
-      <c r="H66" t="inlineStr"/>
     </row>
     <row r="67">
       <c r="A67" t="n">
@@ -1916,21 +1818,20 @@
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>Supralite Os Syp</t>
+          <t>Triavit Plus Cap</t>
         </is>
       </c>
       <c r="C67" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="D67" t="n">
-        <v>309</v>
+        <v>17.34</v>
       </c>
       <c r="E67" t="n">
-        <v>309</v>
+        <v>121.38</v>
       </c>
       <c r="F67" t="inlineStr"/>
       <c r="G67" t="inlineStr"/>
-      <c r="H67" t="inlineStr"/>
     </row>
     <row r="68">
       <c r="A68" t="n">
@@ -1938,43 +1839,41 @@
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>Triavit Plus Cap</t>
+          <t>Voqozon</t>
         </is>
       </c>
       <c r="C68" t="n">
-        <v>7</v>
+        <v>14</v>
       </c>
       <c r="D68" t="n">
-        <v>17.34</v>
+        <v>19.69</v>
       </c>
       <c r="E68" t="n">
-        <v>121.38</v>
+        <v>275.66</v>
       </c>
       <c r="F68" t="inlineStr"/>
       <c r="G68" t="inlineStr"/>
-      <c r="H68" t="inlineStr"/>
     </row>
     <row r="69">
       <c r="A69" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>Voqozon</t>
+          <t>Administrative Charges</t>
         </is>
       </c>
       <c r="C69" t="n">
-        <v>14</v>
+        <v>1</v>
       </c>
       <c r="D69" t="n">
-        <v>19.69</v>
+        <v>55</v>
       </c>
       <c r="E69" t="n">
-        <v>275.66</v>
+        <v>55</v>
       </c>
       <c r="F69" t="inlineStr"/>
       <c r="G69" t="inlineStr"/>
-      <c r="H69" t="inlineStr"/>
     </row>
     <row r="70">
       <c r="A70" t="n">
@@ -1982,21 +1881,20 @@
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>Administrative Charges</t>
+          <t>Admission</t>
         </is>
       </c>
       <c r="C70" t="n">
         <v>1</v>
       </c>
       <c r="D70" t="n">
-        <v>55</v>
+        <v>220</v>
       </c>
       <c r="E70" t="n">
-        <v>55</v>
+        <v>220</v>
       </c>
       <c r="F70" t="inlineStr"/>
       <c r="G70" t="inlineStr"/>
-      <c r="H70" t="inlineStr"/>
     </row>
     <row r="71">
       <c r="A71" t="n">
@@ -2004,21 +1902,20 @@
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>Admission</t>
+          <t>Bed Charges</t>
         </is>
       </c>
       <c r="C71" t="n">
         <v>1</v>
       </c>
       <c r="D71" t="n">
-        <v>220</v>
+        <v>4620</v>
       </c>
       <c r="E71" t="n">
-        <v>220</v>
+        <v>4620</v>
       </c>
       <c r="F71" t="inlineStr"/>
       <c r="G71" t="inlineStr"/>
-      <c r="H71" t="inlineStr"/>
     </row>
     <row r="72">
       <c r="A72" t="n">
@@ -2026,21 +1923,20 @@
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>Bed Charges</t>
+          <t>Dietetics Department</t>
         </is>
       </c>
       <c r="C72" t="n">
         <v>1</v>
       </c>
       <c r="D72" t="n">
-        <v>4620</v>
+        <v>110</v>
       </c>
       <c r="E72" t="n">
-        <v>4620</v>
+        <v>110</v>
       </c>
       <c r="F72" t="inlineStr"/>
       <c r="G72" t="inlineStr"/>
-      <c r="H72" t="inlineStr"/>
     </row>
     <row r="73">
       <c r="A73" t="n">
@@ -2048,21 +1944,20 @@
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>Dietetics Department</t>
+          <t>Doctors Visit Charge</t>
         </is>
       </c>
       <c r="C73" t="n">
         <v>1</v>
       </c>
       <c r="D73" t="n">
-        <v>110</v>
+        <v>330</v>
       </c>
       <c r="E73" t="n">
-        <v>110</v>
+        <v>330</v>
       </c>
       <c r="F73" t="inlineStr"/>
       <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="n">
@@ -2070,21 +1965,20 @@
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>Doctors Visit Charge</t>
+          <t>Laboratory</t>
         </is>
       </c>
       <c r="C74" t="n">
         <v>1</v>
       </c>
       <c r="D74" t="n">
-        <v>330</v>
+        <v>7733</v>
       </c>
       <c r="E74" t="n">
-        <v>330</v>
+        <v>7733</v>
       </c>
       <c r="F74" t="inlineStr"/>
       <c r="G74" t="inlineStr"/>
-      <c r="H74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="n">
@@ -2092,21 +1986,20 @@
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>Laboratory</t>
+          <t>Medicine Charges</t>
         </is>
       </c>
       <c r="C75" t="n">
         <v>1</v>
       </c>
       <c r="D75" t="n">
-        <v>7733</v>
+        <v>20217.4</v>
       </c>
       <c r="E75" t="n">
-        <v>7733</v>
+        <v>20217.4</v>
       </c>
       <c r="F75" t="inlineStr"/>
       <c r="G75" t="inlineStr"/>
-      <c r="H75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="n">
@@ -2114,21 +2007,20 @@
       </c>
       <c r="B76" t="inlineStr">
         <is>
-          <t>Medicine Charges</t>
+          <t>Nursing Charges</t>
         </is>
       </c>
       <c r="C76" t="n">
         <v>1</v>
       </c>
       <c r="D76" t="n">
-        <v>20217.4</v>
+        <v>660</v>
       </c>
       <c r="E76" t="n">
-        <v>20217.4</v>
+        <v>660</v>
       </c>
       <c r="F76" t="inlineStr"/>
       <c r="G76" t="inlineStr"/>
-      <c r="H76" t="inlineStr"/>
     </row>
     <row r="77">
       <c r="A77" t="n">
@@ -2136,21 +2028,20 @@
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>Nursing Charges</t>
+          <t>Procedure/Service Charge</t>
         </is>
       </c>
       <c r="C77" t="n">
         <v>1</v>
       </c>
       <c r="D77" t="n">
-        <v>660</v>
+        <v>220</v>
       </c>
       <c r="E77" t="n">
-        <v>660</v>
+        <v>220</v>
       </c>
       <c r="F77" t="inlineStr"/>
       <c r="G77" t="inlineStr"/>
-      <c r="H77" t="inlineStr"/>
     </row>
     <row r="78">
       <c r="A78" t="n">
@@ -2158,43 +2049,20 @@
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>Procedure/Service Charge</t>
+          <t>Radiology</t>
         </is>
       </c>
       <c r="C78" t="n">
         <v>1</v>
       </c>
       <c r="D78" t="n">
-        <v>220</v>
+        <v>341</v>
       </c>
       <c r="E78" t="n">
-        <v>220</v>
+        <v>341</v>
       </c>
       <c r="F78" t="inlineStr"/>
       <c r="G78" t="inlineStr"/>
-      <c r="H78" t="inlineStr"/>
-    </row>
-    <row r="79">
-      <c r="A79" t="n">
-        <v>5</v>
-      </c>
-      <c r="B79" t="inlineStr">
-        <is>
-          <t>Radiology</t>
-        </is>
-      </c>
-      <c r="C79" t="n">
-        <v>1</v>
-      </c>
-      <c r="D79" t="n">
-        <v>341</v>
-      </c>
-      <c r="E79" t="n">
-        <v>341</v>
-      </c>
-      <c r="F79" t="inlineStr"/>
-      <c r="G79" t="inlineStr"/>
-      <c r="H79" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>